<commit_message>
Update description modalité d'évaluation e84a6ca859ede62255dc1c7a9994c7d746607eb6
</commit_message>
<xml_diff>
--- a/420-contenu-fhir---mise-à-jour-de-lévaluation/ig/StructureDefinition-tddui-assessment-method.xlsx
+++ b/420-contenu-fhir---mise-à-jour-de-lévaluation/ig/StructureDefinition-tddui-assessment-method.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-23T08:45:40+00:00</t>
+    <t>2026-02-23T08:50:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Mode d'évaluation.</t>
+    <t>Mode d'évaluation, texte libre permettant de mettre le contexte de l'évaluation.</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>